<commit_message>
Update manifest template layout to match latest Amazon upload format.
Replace template.xlsx with the current Amazon reference and preserve default owner row spacing and formatting in generated manifests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mthom\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224D74AD-0820-4E2B-90AA-03541B323573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664BDF2B-95BA-4558-AD53-08C769F1F519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-120" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="88">
   <si>
     <t>How to use this Send to Amazon file upload</t>
   </si>
@@ -76,14 +76,10 @@
     <t>Default prep owner</t>
   </si>
   <si>
-    <t>Choose Seller if your units will be prepped before they arrive at the fulfillment center. Choose Amazon to opt in to the FBA Preparation Service.
-If no prep is required, choose Seller.</t>
-  </si>
-  <si>
-    <t>Amazon, Seller</t>
-  </si>
-  <si>
-    <t>Amazon</t>
+    <t>You must prep your products before sending them to our facilities as we do not offer prep services.</t>
+  </si>
+  <si>
+    <t>Seller</t>
   </si>
   <si>
     <t>Required</t>
@@ -95,11 +91,7 @@
     <t>Default labeling owner</t>
   </si>
   <si>
-    <t>Choose Seller if your units will be labeled before they arrive at the fulfillment center. Choose Amazon to opt in to the FBA Label Service. 
-Labeling with an Amazon barcode may not be required if your inventory is tracked using a manufacturer barcode. If no label is required, choose Seller.</t>
-  </si>
-  <si>
-    <t>Seller</t>
+    <t>You must add a barcode to your products before sending them to our facilities as we do not offer labeling services. Labeling with an Amazon barcode may not be required if your inventory is tracked using a manufacturer barcode.</t>
   </si>
   <si>
     <t>Merchant SKU</t>
@@ -123,30 +115,18 @@
     <t>A whole number that is 1 or greater</t>
   </si>
   <si>
-    <t>Prep owner</t>
-  </si>
-  <si>
-    <t>If the prep owner for the MSKU is different from the default prep owner, fill out this column. Otherwise leave it empty.</t>
+    <t>Expiration date</t>
+  </si>
+  <si>
+    <t>If your SKU requires an expiration date, enter the date in MM/DD/YYYY format. If your SKU doesn't require an expiration date, or if you aren't sure if your SKU needs one, leave this column empty. If your MSKU has multiple expiration dates, enter up to four packing lines with unique expiration dates in separate rows.</t>
+  </si>
+  <si>
+    <t>Date in MM/DD/YYYY format</t>
   </si>
   <si>
     <t>Optional</t>
   </si>
   <si>
-    <t>Labeling owner</t>
-  </si>
-  <si>
-    <t>If the labeling owner for the MSKU is different from the default labeling owner, fill out this column. Otherwise leave it empty.</t>
-  </si>
-  <si>
-    <t>Expiration date</t>
-  </si>
-  <si>
-    <t>If your SKU requires an expiration date, enter the date in MM/DD/YYYY format. If your SKU doesn't require an expiration date, or if you aren't sure if your SKU needs one, leave this column empty. If your MSKU has multiple expiration dates, enter up to four packing lines with unique expiration dates in separate rows.</t>
-  </si>
-  <si>
-    <t>Date in MM/DD/YYYY format</t>
-  </si>
-  <si>
     <t>This field is displayed only if you choose to include expiration date in the template. </t>
   </si>
   <si>
@@ -243,31 +223,73 @@
     <t>MyCaseSKU005</t>
   </si>
   <si>
-    <t>842814004580</t>
-  </si>
-  <si>
-    <t>842814004719</t>
-  </si>
-  <si>
-    <t>842814004726</t>
-  </si>
-  <si>
-    <t>842814004733</t>
-  </si>
-  <si>
-    <t>840207113376</t>
-  </si>
-  <si>
-    <t>840207113383</t>
-  </si>
-  <si>
-    <t>840207113390</t>
-  </si>
-  <si>
-    <t>840207113406</t>
-  </si>
-  <si>
-    <t>840207160493</t>
+    <t>195084972715-FNSKU</t>
+  </si>
+  <si>
+    <t>199230226660-FNSKU</t>
+  </si>
+  <si>
+    <t>199230226219-FNSKU</t>
+  </si>
+  <si>
+    <t>199230239936-FNSKU</t>
+  </si>
+  <si>
+    <t>199230246217-FNSKU</t>
+  </si>
+  <si>
+    <t>199230238298-FNSKU</t>
+  </si>
+  <si>
+    <t>199230238342-FNSKU</t>
+  </si>
+  <si>
+    <t>199230226677-FNSKU</t>
+  </si>
+  <si>
+    <t>195084972708-FNSKU</t>
+  </si>
+  <si>
+    <t>199230122498-FNSKU</t>
+  </si>
+  <si>
+    <t>199230239929-FNSKU</t>
+  </si>
+  <si>
+    <t>199230246224-FNSKU</t>
+  </si>
+  <si>
+    <t>199230246200-FNSKU</t>
+  </si>
+  <si>
+    <t>195084442102-FNSKU</t>
+  </si>
+  <si>
+    <t>199230226653-FNSKU</t>
+  </si>
+  <si>
+    <t>199230228299-FNSKU</t>
+  </si>
+  <si>
+    <t>199230123785-FNSKU</t>
+  </si>
+  <si>
+    <t>199230227995-FNSKU</t>
+  </si>
+  <si>
+    <t>199230218696-FNSKU</t>
+  </si>
+  <si>
+    <t>199230228244-FNSKU</t>
+  </si>
+  <si>
+    <t>199230226110-FNSKU</t>
+  </si>
+  <si>
+    <t>199230245142-FNSKU</t>
+  </si>
+  <si>
+    <t>199230224734-FNSKU</t>
   </si>
 </sst>
 </file>
@@ -388,22 +410,18 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="13"/>
       <name val="Amazon Ember"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="20"/>
       <name val="Amazon Ember"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <name val="Amazon Ember"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -691,7 +709,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -709,7 +727,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -754,6 +771,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -793,8 +813,14 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -812,28 +838,28 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1182,57 +1208,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="156" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="25.95" customHeight="1">
-      <c r="A1" s="45" t="s">
+    <row r="1" spans="1:1" ht="26.1" customHeight="1">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="19.05" customHeight="1">
-      <c r="A2" s="46" t="s">
+    <row r="2" spans="1:1" ht="18.95" customHeight="1">
+      <c r="A2" s="48" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="36" customHeight="1">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="49" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="19.05" customHeight="1">
-      <c r="A4" s="46" t="s">
+    <row r="4" spans="1:1" ht="18.95" customHeight="1">
+      <c r="A4" s="48" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="36" customHeight="1">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="49" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="19.05" customHeight="1">
-      <c r="A6" s="46" t="s">
+    <row r="6" spans="1:1" ht="18.95" customHeight="1">
+      <c r="A6" s="48" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="36" customHeight="1">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="50" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="19.95" customHeight="1" thickTop="1">
-      <c r="A8" s="46" t="s">
+    <row r="8" spans="1:1" ht="20.100000000000001" customHeight="1" thickTop="1">
+      <c r="A8" s="48" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="126" customHeight="1">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="50" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="16.95" customHeight="1" thickTop="1"/>
+    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1242,14 +1268,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
     <col min="2" max="2" width="61.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.19921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.125" style="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="1" customWidth="1"/>
     <col min="5" max="5" width="27" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.796875" style="21" customWidth="1"/>
+    <col min="6" max="6" width="25.875" style="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1">
@@ -1268,274 +1294,240 @@
       <c r="E1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="54" customHeight="1">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="52" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="72" customHeight="1">
+      <c r="A3" s="25" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="72" customHeight="1">
-      <c r="A3" s="26" t="s">
+      <c r="B3" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="56"/>
+    </row>
+    <row r="4" spans="1:6" ht="108" customHeight="1">
+      <c r="A4" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="14" t="s">
+      <c r="B4" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="53"/>
-    </row>
-    <row r="4" spans="1:6" ht="108" customHeight="1">
-      <c r="A4" s="26" t="s">
+      <c r="C4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="D4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="E4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="19"/>
+    </row>
+    <row r="5" spans="1:6" ht="36" customHeight="1">
+      <c r="A5" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="20"/>
-    </row>
-    <row r="5" spans="1:6" ht="36" customHeight="1">
-      <c r="A5" s="27" t="s">
+      <c r="C5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="D5" s="13">
+        <v>1</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="16"/>
+    </row>
+    <row r="6" spans="1:6" ht="36" customHeight="1">
+      <c r="A6" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="B6" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="14">
-        <v>1</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="17"/>
-    </row>
-    <row r="6" spans="1:6" ht="36" customHeight="1">
-      <c r="A6" s="28" t="s">
+      <c r="C6" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="D6" s="24">
+        <v>47771</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="20"/>
+      <c r="C7" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="90" customHeight="1">
-      <c r="A8" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="25">
-        <v>47771</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="18" t="s">
+      <c r="A8" s="27" t="s">
         <v>39</v>
       </c>
+      <c r="B8" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="13">
+        <v>40</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="55" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="72" customHeight="1">
-      <c r="A9" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="A9" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>44</v>
-      </c>
+      <c r="C9" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="13">
+        <v>7</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="57"/>
     </row>
     <row r="10" spans="1:6" ht="54" customHeight="1">
       <c r="A10" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="C10" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="14">
-        <v>40</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="52" t="s">
-        <v>47</v>
-      </c>
+      <c r="D10" s="13">
+        <v>15.5</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="57"/>
     </row>
     <row r="11" spans="1:6" ht="36" customHeight="1">
       <c r="A11" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="C11" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="13">
+        <v>15.5</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="57"/>
+    </row>
+    <row r="12" spans="1:6" ht="18" customHeight="1">
+      <c r="A12" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="14">
-        <v>7</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="54"/>
-    </row>
-    <row r="12" spans="1:6" ht="18" customHeight="1">
-      <c r="A12" s="29" t="s">
+      <c r="B12" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="C12" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="13">
+        <v>10.75</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="57"/>
+    </row>
+    <row r="13" spans="1:6" ht="18" customHeight="1">
+      <c r="A13" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="14">
-        <v>15.5</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="54"/>
-    </row>
-    <row r="13" spans="1:6" ht="18" customHeight="1">
-      <c r="A13" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="14">
-        <v>15.5</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="54"/>
-    </row>
-    <row r="14" spans="1:6" ht="18" customHeight="1">
-      <c r="A14" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="14">
-        <v>10.75</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="54"/>
-    </row>
-    <row r="15" spans="1:6" ht="18" customHeight="1">
-      <c r="A15" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" s="14">
+      <c r="C13" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="13">
         <v>20.25</v>
       </c>
-      <c r="E15" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="53"/>
-    </row>
+      <c r="E13" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="56"/>
+    </row>
+    <row r="14" spans="1:6" ht="18" customHeight="1"/>
+    <row r="15" spans="1:6" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F2:F3"/>
-    <mergeCell ref="F10:F15"/>
+    <mergeCell ref="F8:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1543,39 +1535,39 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.8"/>
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="28" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.5" style="2" customWidth="1"/>
-    <col min="7" max="7" width="21" style="2" customWidth="1"/>
-    <col min="8" max="8" width="17" style="2" customWidth="1"/>
-    <col min="9" max="9" width="17.5" style="2" customWidth="1"/>
-    <col min="10" max="10" width="20" style="2" customWidth="1"/>
-    <col min="11" max="11" width="11" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="11" style="2"/>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="9.875" customWidth="1"/>
+    <col min="3" max="3" width="33.5" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="20.5" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="6" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A1" s="43" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="44"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="A1" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="45"/>
+    </row>
+    <row r="2" spans="1:10" ht="16.5">
       <c r="A2" s="3"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -1584,10 +1576,14 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+    <row r="3" spans="1:10" ht="16.5">
+      <c r="A3" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -1596,10 +1592,14 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10" ht="18" customHeight="1" thickBot="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+    <row r="4" spans="1:10" ht="16.5">
+      <c r="A4" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -1608,134 +1608,270 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="13"/>
-    </row>
-    <row r="6" spans="1:10" s="37" customFormat="1" ht="37.5" customHeight="1" thickBot="1">
-      <c r="A6" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="35" t="s">
+    <row r="5" spans="1:10" ht="16.5">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" ht="18" customHeight="1" thickBot="1">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="12"/>
+    </row>
+    <row r="8" spans="1:10" s="37" customFormat="1" ht="37.5" customHeight="1" thickBot="1">
+      <c r="A8" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="36" t="s">
+      <c r="D8" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="32" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="60" t="s">
+      <c r="F8" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="36" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="64">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="61">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="60" t="s">
+      <c r="B15" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="60" t="s">
+      <c r="B16" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="60" t="s">
+      <c r="B17" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="B10" s="61">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="60" t="s">
+      <c r="B18" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="60" t="s">
+      <c r="B19" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="60" t="s">
+      <c r="B20" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="60" t="s">
+      <c r="B21" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="61">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="62" t="s">
+      <c r="B22" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="63" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="61">
-        <v>18</v>
+      <c r="B23" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="63" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="63" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="64">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A7:A10">
+  <conditionalFormatting sqref="A9:A12">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A11:A14">
+  <conditionalFormatting sqref="A13:A16">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15">
+  <conditionalFormatting sqref="A17">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1745,38 +1881,38 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.8"/>
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="26.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="2" customWidth="1"/>
-    <col min="3" max="3" width="33.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="28" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.5" style="2" customWidth="1"/>
-    <col min="7" max="7" width="21" style="2" customWidth="1"/>
-    <col min="8" max="8" width="17" style="2" customWidth="1"/>
-    <col min="9" max="9" width="17.5" style="2" customWidth="1"/>
-    <col min="10" max="10" width="20" style="2" customWidth="1"/>
-    <col min="11" max="11" width="11" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="11" style="2"/>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="33.5" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="20.5" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A1" s="55" t="s">
-        <v>64</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="57"/>
-    </row>
-    <row r="2" spans="1:10">
+    <row r="1" spans="1:12" s="5" customFormat="1" ht="28.5" customHeight="1">
+      <c r="A1" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="60"/>
+    </row>
+    <row r="2" spans="1:12" ht="16.5">
       <c r="A2" s="58"/>
       <c r="B2" s="59"/>
       <c r="C2" s="59"/>
@@ -1786,11 +1922,17 @@
       <c r="G2" s="59"/>
       <c r="H2" s="59"/>
       <c r="I2" s="59"/>
-      <c r="J2" s="57"/>
-    </row>
-    <row r="3" spans="1:10" ht="18" customHeight="1" thickBot="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="60"/>
+    </row>
+    <row r="3" spans="1:12" ht="16.5">
+      <c r="A3" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>17</v>
+      </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -1800,249 +1942,277 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10" ht="18" customHeight="1" thickBot="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="23" t="s">
+    <row r="4" spans="1:12" ht="16.5">
+      <c r="A4" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:12" ht="18" customHeight="1" thickBot="1">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:12" ht="18" customHeight="1" thickBot="1">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="10"/>
+      <c r="E6" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="10"/>
+    </row>
+    <row r="7" spans="1:12" s="37" customFormat="1" ht="37.5" customHeight="1" thickBot="1">
+      <c r="A7" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="42" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="16.5">
+      <c r="A8" s="52" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="11"/>
-    </row>
-    <row r="5" spans="1:10" s="37" customFormat="1" ht="37.5" customHeight="1" thickBot="1">
-      <c r="A5" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="38" t="s">
+      <c r="B8" s="52">
+        <v>23</v>
+      </c>
+      <c r="C8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="52"/>
+    </row>
+    <row r="9" spans="1:12" ht="16.5">
+      <c r="A9" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="38" t="s">
+      <c r="B9" s="52">
+        <v>12</v>
+      </c>
+      <c r="C9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
+    </row>
+    <row r="10" spans="1:12" ht="16.5">
+      <c r="A10" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="52">
+        <v>30</v>
+      </c>
+      <c r="C10" s="53">
+        <v>45709</v>
+      </c>
+      <c r="D10" s="23">
+        <v>123456789</v>
+      </c>
+      <c r="E10" s="52">
+        <v>10</v>
+      </c>
+      <c r="F10" s="52">
+        <v>3</v>
+      </c>
+      <c r="G10" s="52">
+        <v>12.5</v>
+      </c>
+      <c r="H10" s="52">
+        <v>12.5</v>
+      </c>
+      <c r="I10" s="52">
+        <v>12.5</v>
+      </c>
+      <c r="J10" s="52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="16.5">
+      <c r="A11" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="52">
+        <v>75</v>
+      </c>
+      <c r="C11" s="53">
+        <v>45709</v>
+      </c>
+      <c r="E11" s="52">
+        <v>15</v>
+      </c>
+      <c r="F11" s="52">
+        <v>5</v>
+      </c>
+      <c r="G11" s="52">
+        <v>14.5</v>
+      </c>
+      <c r="H11" s="52">
+        <v>10</v>
+      </c>
+      <c r="I11" s="52">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J11" s="52">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="16.5">
+      <c r="A12" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="52">
+        <v>80</v>
+      </c>
+      <c r="C12" s="53">
+        <v>45798</v>
+      </c>
+      <c r="E12" s="52">
+        <v>20</v>
+      </c>
+      <c r="F12" s="52">
+        <v>4</v>
+      </c>
+      <c r="G12" s="52">
+        <v>14.5</v>
+      </c>
+      <c r="H12" s="52">
+        <v>10</v>
+      </c>
+      <c r="I12" s="52">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J12" s="52">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A13" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="52">
+        <v>50</v>
+      </c>
+      <c r="C13" s="53">
+        <v>45829</v>
+      </c>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="52"/>
+      <c r="J13" s="52"/>
+    </row>
+    <row r="14" spans="1:12" ht="16.5">
+      <c r="A14" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="H5" s="40" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="J5" s="42" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="50" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="50">
-        <v>23</v>
-      </c>
-      <c r="C6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
-      <c r="J6" s="50"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="50" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="50">
-        <v>12</v>
-      </c>
-      <c r="C7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="50" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="50">
+      <c r="B14" s="52">
         <v>30</v>
       </c>
-      <c r="C8" s="51">
-        <v>45709</v>
-      </c>
-      <c r="D8" s="24">
-        <v>123456789</v>
-      </c>
-      <c r="E8" s="50">
+      <c r="C14" s="52"/>
+      <c r="E14" s="52">
         <v>10</v>
       </c>
-      <c r="F8" s="50">
+      <c r="F14" s="52">
         <v>3</v>
       </c>
-      <c r="G8" s="50">
+      <c r="G14" s="52">
         <v>12.5</v>
       </c>
-      <c r="H8" s="50">
+      <c r="H14" s="52">
         <v>12.5</v>
       </c>
-      <c r="I8" s="50">
+      <c r="I14" s="52">
         <v>12.5</v>
       </c>
-      <c r="J8" s="50">
+      <c r="J14" s="52">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="50" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="50">
+    <row r="15" spans="1:12" ht="16.5">
+      <c r="A15" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="52">
         <v>75</v>
       </c>
-      <c r="C9" s="51">
-        <v>45709</v>
-      </c>
-      <c r="E9" s="50">
+      <c r="C15" s="52"/>
+      <c r="E15" s="52">
         <v>15</v>
       </c>
-      <c r="F9" s="50">
-        <v>5</v>
-      </c>
-      <c r="G9" s="50">
+      <c r="F15" s="52">
+        <v>5</v>
+      </c>
+      <c r="G15" s="52">
         <v>14.5</v>
       </c>
-      <c r="H9" s="50">
+      <c r="H15" s="52">
         <v>10</v>
       </c>
-      <c r="I9" s="50">
+      <c r="I15" s="52">
         <v>8.3000000000000007</v>
       </c>
-      <c r="J9" s="50">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="50" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="50">
-        <v>80</v>
-      </c>
-      <c r="C10" s="51">
-        <v>45798</v>
-      </c>
-      <c r="E10" s="50">
-        <v>20</v>
-      </c>
-      <c r="F10" s="50">
-        <v>4</v>
-      </c>
-      <c r="G10" s="50">
-        <v>14.5</v>
-      </c>
-      <c r="H10" s="50">
-        <v>10</v>
-      </c>
-      <c r="I10" s="50">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="J10" s="50">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="25.05" customHeight="1">
-      <c r="A11" s="50" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" s="50">
-        <v>50</v>
-      </c>
-      <c r="C11" s="51">
-        <v>45829</v>
-      </c>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="50"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="50" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="50">
-        <v>30</v>
-      </c>
-      <c r="C12" s="50"/>
-      <c r="E12" s="50">
-        <v>10</v>
-      </c>
-      <c r="F12" s="50">
-        <v>3</v>
-      </c>
-      <c r="G12" s="50">
-        <v>12.5</v>
-      </c>
-      <c r="H12" s="50">
-        <v>12.5</v>
-      </c>
-      <c r="I12" s="50">
-        <v>12.5</v>
-      </c>
-      <c r="J12" s="50">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="50" t="s">
-        <v>70</v>
-      </c>
-      <c r="B13" s="50">
-        <v>75</v>
-      </c>
-      <c r="C13" s="50"/>
-      <c r="E13" s="50">
-        <v>15</v>
-      </c>
-      <c r="F13" s="50">
-        <v>5</v>
-      </c>
-      <c r="G13" s="50">
-        <v>14.5</v>
-      </c>
-      <c r="H13" s="50">
-        <v>10</v>
-      </c>
-      <c r="I13" s="50">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="J13" s="50">
+      <c r="J15" s="52">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>